<commit_message>
added png versions of images
</commit_message>
<xml_diff>
--- a/8-26 Ewing Gallery Schief.xlsx
+++ b/8-26 Ewing Gallery Schief.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0c1ec16cd9456fc5/Desktop/DH 200/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0c1ec16cd9456fc5/Desktop/DH 200/Schief-Ewing-Gallery/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="103" documentId="11_EE22872F66CAC18352571B75917E9B827B1F9662" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AEFCFCD-2893-4DE6-86C9-7A76523432DE}"/>
   <bookViews>
-    <workbookView xWindow="4770" yWindow="8270" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3190" yWindow="7250" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>